<commit_message>
fix(sync): preserve active versions and reconcile shared work data
</commit_message>
<xml_diff>
--- a/home/data/Material_Inventory.xlsx
+++ b/home/data/Material_Inventory.xlsx
@@ -24725,7 +24725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DE4"/>
+  <dimension ref="A1:DE5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26070,6 +26070,257 @@
         <v>0</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="1" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>중앙지사</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>480</v>
+      </c>
+      <c r="D5" t="n">
+        <v>4.4686</v>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" s="1" t="n">
+        <v>46269.52358722223</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>부장 주진철</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>PAUT MX2(OMNI2-103085)</t>
+        </is>
+      </c>
+      <c r="P5" t="n">
+        <v>4.4686</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>201862</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" t="n">
+        <v>902042</v>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>PAUT</t>
+        </is>
+      </c>
+      <c r="V5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~18:00</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>부장 박광복</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~18:00</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr"/>
+      <c r="AG5" t="inlineStr"/>
+      <c r="AH5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr"/>
+      <c r="AJ5" t="inlineStr"/>
+      <c r="AK5" t="inlineStr"/>
+      <c r="AL5" t="inlineStr"/>
+      <c r="AM5" t="inlineStr"/>
+      <c r="AN5" t="inlineStr"/>
+      <c r="AO5" t="inlineStr"/>
+      <c r="AP5" t="inlineStr"/>
+      <c r="AQ5" t="inlineStr"/>
+      <c r="AR5" t="inlineStr"/>
+      <c r="AS5" t="inlineStr"/>
+      <c r="AT5" t="inlineStr"/>
+      <c r="AU5" t="inlineStr"/>
+      <c r="AV5" t="inlineStr"/>
+      <c r="AW5" t="inlineStr"/>
+      <c r="AX5" t="inlineStr"/>
+      <c r="AY5" t="inlineStr"/>
+      <c r="AZ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG5" t="inlineStr">
+        <is>
+          <t>81도5958 (스타렉스)</t>
+        </is>
+      </c>
+      <c r="BH5" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="BI5" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함</t>
+        </is>
+      </c>
+      <c r="BJ5" t="inlineStr"/>
+      <c r="BK5" t="inlineStr"/>
+      <c r="BL5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM5" t="inlineStr"/>
+      <c r="BN5" t="inlineStr">
+        <is>
+          <t>한국지역난방공사 중앙지사</t>
+        </is>
+      </c>
+      <c r="BO5" t="inlineStr"/>
+      <c r="BP5" t="inlineStr"/>
+      <c r="BQ5" t="inlineStr"/>
+      <c r="BR5" t="inlineStr"/>
+      <c r="BS5" t="inlineStr"/>
+      <c r="BT5" t="inlineStr"/>
+      <c r="BU5" t="inlineStr"/>
+      <c r="BV5" t="inlineStr">
+        <is>
+          <t>Pipe</t>
+        </is>
+      </c>
+      <c r="BW5" t="inlineStr"/>
+      <c r="BX5" t="inlineStr"/>
+      <c r="BY5" t="inlineStr"/>
+      <c r="BZ5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="CA5" t="inlineStr"/>
+      <c r="CB5" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="CC5" t="inlineStr">
+        <is>
+          <t>300A 이상 (1.0)</t>
+        </is>
+      </c>
+      <c r="CD5" t="inlineStr"/>
+      <c r="CE5" t="inlineStr"/>
+      <c r="CF5" t="inlineStr"/>
+      <c r="CG5" t="n">
+        <v>1</v>
+      </c>
+      <c r="CH5" t="n">
+        <v>4.4686</v>
+      </c>
+      <c r="CI5" t="n">
+        <v>167836</v>
+      </c>
+      <c r="CJ5" t="n">
+        <v>291352</v>
+      </c>
+      <c r="CK5" t="n">
+        <v>320487</v>
+      </c>
+      <c r="CL5" t="n">
+        <v>122367</v>
+      </c>
+      <c r="CM5" t="inlineStr"/>
+      <c r="CN5" t="inlineStr"/>
+      <c r="CO5" t="inlineStr"/>
+      <c r="CP5" t="inlineStr"/>
+      <c r="CQ5" t="inlineStr"/>
+      <c r="CR5" t="inlineStr"/>
+      <c r="CS5" t="inlineStr"/>
+      <c r="CT5" t="inlineStr"/>
+      <c r="CU5" t="inlineStr"/>
+      <c r="CV5" t="inlineStr"/>
+      <c r="CW5" t="inlineStr">
+        <is>
+          <t>ORI</t>
+        </is>
+      </c>
+      <c r="CX5" t="n">
+        <v>2</v>
+      </c>
+      <c r="CY5" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ5" t="inlineStr">
+        <is>
+          <t>700A</t>
+        </is>
+      </c>
+      <c r="DA5" t="inlineStr">
+        <is>
+          <t>열배관</t>
+        </is>
+      </c>
+      <c r="DB5" t="inlineStr"/>
+      <c r="DC5" t="inlineStr"/>
+      <c r="DD5" t="inlineStr"/>
+      <c r="DE5" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>